<commit_message>
def remainder_message(i) This Funcation Message Some Issue Fix
</commit_message>
<xml_diff>
--- a/gemini bot - Copy (2)/whatsapp_bot - Copy/reports/Bikash_Beherasales_report.xlsx
+++ b/gemini bot - Copy (2)/whatsapp_bot - Copy/reports/Bikash_Beherasales_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB97"/>
+  <dimension ref="A1:BB99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1661,7 +1661,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1975,7 +1975,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2856,7 +2856,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -3016,7 +3016,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -3160,7 +3160,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -3290,7 +3290,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -3430,7 +3430,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -3570,7 +3570,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -3710,7 +3710,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -3850,7 +3850,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -3990,7 +3990,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -4130,7 +4130,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -4294,7 +4294,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -4424,7 +4424,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -4589,7 +4589,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -4753,7 +4753,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -4917,7 +4917,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -5213,7 +5213,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -5353,7 +5353,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -5493,7 +5493,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -5753,7 +5753,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -5883,7 +5883,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -6027,7 +6027,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -6149,7 +6149,7 @@
       </c>
       <c r="AM38" t="inlineStr">
         <is>
-          <t>DSD-2627/00958,DSD-2627/01026</t>
+          <t>DSD-2627/01026,DSD-2627/00958</t>
         </is>
       </c>
       <c r="AN38" t="inlineStr">
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -6376,7 +6376,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -6521,7 +6521,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -6666,7 +6666,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -6850,7 +6850,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -6988,7 +6988,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -7143,7 +7143,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -7256,7 +7256,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -7401,7 +7401,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -7546,7 +7546,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -7730,7 +7730,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -7914,7 +7914,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -8099,7 +8099,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -8245,7 +8245,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -8376,7 +8376,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -8507,7 +8507,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -8637,7 +8637,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -8782,7 +8782,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -8927,7 +8927,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -9034,9 +9034,19 @@
       <c r="AI57" t="n">
         <v>281.5</v>
       </c>
-      <c r="AJ57" t="inlineStr"/>
-      <c r="AK57" t="inlineStr"/>
-      <c r="AL57" t="inlineStr"/>
+      <c r="AJ57" t="inlineStr">
+        <is>
+          <t>DJC-2627/10249</t>
+        </is>
+      </c>
+      <c r="AK57" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="AL57" t="n">
+        <v>259.75</v>
+      </c>
       <c r="AM57" t="inlineStr"/>
       <c r="AN57" t="inlineStr"/>
       <c r="AO57" t="inlineStr"/>
@@ -9082,7 +9092,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -9226,7 +9236,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -9370,7 +9380,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -9514,7 +9524,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -9658,7 +9668,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -9802,7 +9812,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -9966,7 +9976,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -10073,9 +10083,19 @@
       <c r="AI64" t="n">
         <v>205</v>
       </c>
-      <c r="AJ64" t="inlineStr"/>
-      <c r="AK64" t="inlineStr"/>
-      <c r="AL64" t="inlineStr"/>
+      <c r="AJ64" t="inlineStr">
+        <is>
+          <t>DJC-2627/10249</t>
+        </is>
+      </c>
+      <c r="AK64" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="AL64" t="n">
+        <v>201.5</v>
+      </c>
       <c r="AM64" t="inlineStr"/>
       <c r="AN64" t="inlineStr"/>
       <c r="AO64" t="inlineStr"/>
@@ -10121,7 +10141,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -10228,9 +10248,19 @@
       <c r="AI65" t="n">
         <v>94</v>
       </c>
-      <c r="AJ65" t="inlineStr"/>
-      <c r="AK65" t="inlineStr"/>
-      <c r="AL65" t="inlineStr"/>
+      <c r="AJ65" t="inlineStr">
+        <is>
+          <t>DJC-2627/10249</t>
+        </is>
+      </c>
+      <c r="AK65" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="AL65" t="n">
+        <v>90.75</v>
+      </c>
       <c r="AM65" t="inlineStr"/>
       <c r="AN65" t="inlineStr"/>
       <c r="AO65" t="inlineStr"/>
@@ -10276,7 +10306,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -10430,7 +10460,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -10560,7 +10590,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -10745,7 +10775,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -10889,7 +10919,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -11019,7 +11049,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -11127,7 +11157,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -11269,7 +11299,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -11376,9 +11406,19 @@
       <c r="AI73" t="n">
         <v>102</v>
       </c>
-      <c r="AJ73" t="inlineStr"/>
-      <c r="AK73" t="inlineStr"/>
-      <c r="AL73" t="inlineStr"/>
+      <c r="AJ73" t="inlineStr">
+        <is>
+          <t>DJC-2627/10249</t>
+        </is>
+      </c>
+      <c r="AK73" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="AL73" t="n">
+        <v>98</v>
+      </c>
       <c r="AM73" t="inlineStr"/>
       <c r="AN73" t="inlineStr"/>
       <c r="AO73" t="inlineStr"/>
@@ -11424,7 +11464,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -11562,7 +11602,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -11692,7 +11732,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -11823,7 +11863,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -11961,7 +12001,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -12099,7 +12139,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -12237,7 +12277,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -12375,7 +12415,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -12503,7 +12543,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -12633,7 +12673,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -12763,7 +12803,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -12893,7 +12933,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -13023,7 +13063,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -13161,7 +13201,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -13174,10 +13214,10 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>800</v>
+        <v>670</v>
       </c>
       <c r="G87" t="n">
-        <v>0</v>
+        <v>657</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -13229,19 +13269,27 @@
       </c>
       <c r="AJ87" t="inlineStr">
         <is>
-          <t>DJC-2627/10237,DJC-2627/10238,DJC-2627/10239,DJC-2627/10240,DJC-2627/10241,DJC-2627/10242</t>
+          <t>DJC-2627/10237,DJC-2627/10238,DJC-2627/10239,DJC-2627/10240,DJC-2627/10241,DJC-2627/10242,DJC-2627/10251</t>
         </is>
       </c>
       <c r="AK87" t="inlineStr">
         <is>
-          <t>2026-09-26,2026-09-26,2026-09-26,2026-09-26,2026-09-26,2026-09-26</t>
+          <t>2026-09-26,2026-09-26,2026-09-26,2026-09-26,2026-09-26,2026-09-26,2026-09-28</t>
         </is>
       </c>
       <c r="AL87" t="n">
-        <v>578</v>
-      </c>
-      <c r="AM87" t="inlineStr"/>
-      <c r="AN87" t="inlineStr"/>
+        <v>657</v>
+      </c>
+      <c r="AM87" t="inlineStr">
+        <is>
+          <t>DSD-2627/01032</t>
+        </is>
+      </c>
+      <c r="AN87" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="AO87" t="inlineStr"/>
       <c r="AP87" t="inlineStr"/>
       <c r="AQ87" t="n">
@@ -13264,7 +13312,9 @@
       <c r="AX87" t="inlineStr"/>
       <c r="AY87" t="inlineStr"/>
       <c r="AZ87" t="inlineStr"/>
-      <c r="BA87" t="inlineStr"/>
+      <c r="BA87" t="n">
+        <v>2</v>
+      </c>
       <c r="BB87" t="inlineStr"/>
     </row>
     <row r="88">
@@ -13279,7 +13329,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -13400,46 +13450,50 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Lohia Overseas LLP</t>
+          <t>K M ENTERPRISE</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>['ESO-2627/01328']</t>
+          <t>['DSO-2627/01204']</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>177</v>
+        <v>775</v>
       </c>
       <c r="G89" t="n">
-        <v>100.5</v>
+        <v>0</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Kolkata</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr"/>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>ORDER BY BIKASH BHAI(WG)</t>
+        </is>
+      </c>
       <c r="J89" t="inlineStr">
         <is>
           <t>Bikash Behera</t>
         </is>
       </c>
       <c r="K89" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr"/>
@@ -13475,41 +13529,15 @@
       <c r="AI89" t="n">
         <v>0</v>
       </c>
-      <c r="AJ89" t="inlineStr">
-        <is>
-          <t>EJC-2627/04018,EJC-2627/04019,EJC-2627/04020,EJC-2627/04021,EJC-2627/04022</t>
-        </is>
-      </c>
-      <c r="AK89" t="inlineStr">
-        <is>
-          <t>2026-07-11,2026-07-11,2026-07-11,2026-07-11,2026-07-11</t>
-        </is>
-      </c>
-      <c r="AL89" t="n">
-        <v>100.5</v>
-      </c>
-      <c r="AM89" t="inlineStr">
-        <is>
-          <t>ESD-2627/01690</t>
-        </is>
-      </c>
-      <c r="AN89" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="AO89" t="inlineStr">
-        <is>
-          <t>ESI-2627/01673</t>
-        </is>
-      </c>
-      <c r="AP89" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
+      <c r="AJ89" t="inlineStr"/>
+      <c r="AK89" t="inlineStr"/>
+      <c r="AL89" t="inlineStr"/>
+      <c r="AM89" t="inlineStr"/>
+      <c r="AN89" t="inlineStr"/>
+      <c r="AO89" t="inlineStr"/>
+      <c r="AP89" t="inlineStr"/>
       <c r="AQ89" t="n">
-        <v>100.5</v>
+        <v>0</v>
       </c>
       <c r="AR89" t="inlineStr">
         <is>
@@ -13528,46 +13556,42 @@
       <c r="AX89" t="inlineStr"/>
       <c r="AY89" t="inlineStr"/>
       <c r="AZ89" t="inlineStr"/>
-      <c r="BA89" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB89" t="n">
-        <v>0</v>
-      </c>
+      <c r="BA89" t="inlineStr"/>
+      <c r="BB89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Bee Kay Textiles</t>
+          <t>Lohia Overseas LLP</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>['PSO-2627/01171']</t>
+          <t>['ESO-2627/01328']</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>137</v>
+        <v>79</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>21</v>
+        <v>177</v>
       </c>
       <c r="G90" t="n">
-        <v>0</v>
+        <v>100.5</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Jalandhar City</t>
+          <t>Kolkata</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -13577,7 +13601,7 @@
         </is>
       </c>
       <c r="K90" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr"/>
@@ -13613,15 +13637,41 @@
       <c r="AI90" t="n">
         <v>0</v>
       </c>
-      <c r="AJ90" t="inlineStr"/>
-      <c r="AK90" t="inlineStr"/>
-      <c r="AL90" t="inlineStr"/>
-      <c r="AM90" t="inlineStr"/>
-      <c r="AN90" t="inlineStr"/>
-      <c r="AO90" t="inlineStr"/>
-      <c r="AP90" t="inlineStr"/>
+      <c r="AJ90" t="inlineStr">
+        <is>
+          <t>EJC-2627/04018,EJC-2627/04019,EJC-2627/04020,EJC-2627/04021,EJC-2627/04022</t>
+        </is>
+      </c>
+      <c r="AK90" t="inlineStr">
+        <is>
+          <t>2026-07-11,2026-07-11,2026-07-11,2026-07-11,2026-07-11</t>
+        </is>
+      </c>
+      <c r="AL90" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="AM90" t="inlineStr">
+        <is>
+          <t>ESD-2627/01690</t>
+        </is>
+      </c>
+      <c r="AN90" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="AO90" t="inlineStr">
+        <is>
+          <t>ESI-2627/01673</t>
+        </is>
+      </c>
+      <c r="AP90" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
       <c r="AQ90" t="n">
-        <v>0</v>
+        <v>100.5</v>
       </c>
       <c r="AR90" t="inlineStr">
         <is>
@@ -13640,31 +13690,35 @@
       <c r="AX90" t="inlineStr"/>
       <c r="AY90" t="inlineStr"/>
       <c r="AZ90" t="inlineStr"/>
-      <c r="BA90" t="inlineStr"/>
-      <c r="BB90" t="inlineStr"/>
+      <c r="BA90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Casa De Gorras Ladies Wears Fashion Llp</t>
+          <t>Bee Kay Textiles</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>['PSO-2627/04010']</t>
+          <t>['PSO-2627/01171']</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>6</v>
+        <v>138</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="F91" t="n">
@@ -13675,21 +13729,17 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Mumbai</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SAMPLE DONO SATH ME JAYEGA </t>
-        </is>
-      </c>
+          <t>Jalandhar City</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr">
         <is>
           <t>Bikash Behera</t>
         </is>
       </c>
       <c r="K91" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>
@@ -13705,48 +13755,20 @@
       <c r="U91" t="n">
         <v>0</v>
       </c>
-      <c r="V91" t="inlineStr">
-        <is>
-          <t>PJO-2627/04408,PJO-2627/04409-1</t>
-        </is>
-      </c>
-      <c r="W91" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="X91" t="inlineStr">
-        <is>
-          <t>RFD-Musline Heavy 63 T,RFD-Musline Heavy MP (EV),RFD-MUSLINE HEAVY V</t>
-        </is>
-      </c>
+      <c r="V91" t="inlineStr"/>
+      <c r="W91" t="inlineStr"/>
+      <c r="X91" t="inlineStr"/>
       <c r="Y91" t="n">
-        <v>21</v>
-      </c>
-      <c r="Z91" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Z91" t="inlineStr"/>
       <c r="AA91" t="inlineStr"/>
       <c r="AB91" t="inlineStr"/>
-      <c r="AC91" t="inlineStr">
-        <is>
-          <t>Gokul Texprints Pvt. Ltd. (Sachin),Gokul Texprints Pvt. Ltd. (Sachin)</t>
-        </is>
-      </c>
-      <c r="AD91" t="inlineStr">
-        <is>
-          <t>RVI-2627/07397,RVI-2627/07402</t>
-        </is>
-      </c>
-      <c r="AE91" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+      <c r="AC91" t="inlineStr"/>
+      <c r="AD91" t="inlineStr"/>
+      <c r="AE91" t="inlineStr"/>
       <c r="AF91" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="AG91" t="inlineStr"/>
       <c r="AH91" t="inlineStr"/>
@@ -13774,15 +13796,11 @@
           <t>Bikash Behera</t>
         </is>
       </c>
-      <c r="AU91" t="n">
-        <v>1</v>
-      </c>
+      <c r="AU91" t="inlineStr"/>
       <c r="AV91" t="inlineStr"/>
       <c r="AW91" t="inlineStr"/>
       <c r="AX91" t="inlineStr"/>
-      <c r="AY91" t="n">
-        <v>0</v>
-      </c>
+      <c r="AY91" t="inlineStr"/>
       <c r="AZ91" t="inlineStr"/>
       <c r="BA91" t="inlineStr"/>
       <c r="BB91" t="inlineStr"/>
@@ -13799,7 +13817,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -13970,46 +13988,50 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Manisha Fabrics (Raipur)</t>
+          <t>Casa De Gorras Ladies Wears Fashion Llp</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>['PSO-2627/04106']</t>
+          <t>['PSO-2627/04010']</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>140</v>
+        <v>21</v>
       </c>
       <c r="G93" t="n">
         <v>0</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Raipur</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr"/>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAMPLE DONO SATH ME JAYEGA </t>
+        </is>
+      </c>
       <c r="J93" t="inlineStr">
         <is>
           <t>Bikash Behera</t>
         </is>
       </c>
       <c r="K93" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr"/>
@@ -14027,21 +14049,21 @@
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>PJO-2627/04514</t>
+          <t>PJO-2627/04408,PJO-2627/04409-1</t>
         </is>
       </c>
       <c r="W93" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>RFD-Natural Crepe (M)</t>
+          <t>RFD-Musline Heavy 63 T,RFD-Musline Heavy MP (EV),RFD-MUSLINE HEAVY V</t>
         </is>
       </c>
       <c r="Y93" t="n">
-        <v>140</v>
+        <v>21</v>
       </c>
       <c r="Z93" t="inlineStr">
         <is>
@@ -14050,11 +14072,23 @@
       </c>
       <c r="AA93" t="inlineStr"/>
       <c r="AB93" t="inlineStr"/>
-      <c r="AC93" t="inlineStr"/>
-      <c r="AD93" t="inlineStr"/>
-      <c r="AE93" t="inlineStr"/>
+      <c r="AC93" t="inlineStr">
+        <is>
+          <t>Gokul Texprints Pvt. Ltd. (Sachin),Gokul Texprints Pvt. Ltd. (Sachin)</t>
+        </is>
+      </c>
+      <c r="AD93" t="inlineStr">
+        <is>
+          <t>RVI-2627/07397,RVI-2627/07402</t>
+        </is>
+      </c>
+      <c r="AE93" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="AF93" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="AG93" t="inlineStr"/>
       <c r="AH93" t="inlineStr"/>
@@ -14083,12 +14117,14 @@
         </is>
       </c>
       <c r="AU93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV93" t="inlineStr"/>
       <c r="AW93" t="inlineStr"/>
       <c r="AX93" t="inlineStr"/>
-      <c r="AY93" t="inlineStr"/>
+      <c r="AY93" t="n">
+        <v>0</v>
+      </c>
       <c r="AZ93" t="inlineStr"/>
       <c r="BA93" t="inlineStr"/>
       <c r="BB93" t="inlineStr"/>
@@ -14101,11 +14137,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>['PSO-2627/04107']</t>
+          <t>['PSO-2627/04106']</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -14118,7 +14154,7 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>620</v>
+        <v>140</v>
       </c>
       <c r="G94" t="n">
         <v>0</v>
@@ -14153,7 +14189,7 @@
       </c>
       <c r="V94" t="inlineStr">
         <is>
-          <t>PJO-2627/04513-1</t>
+          <t>PJO-2627/04514</t>
         </is>
       </c>
       <c r="W94" t="inlineStr">
@@ -14163,11 +14199,11 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>RFD-Satin Bemberg New</t>
+          <t>RFD-Natural Crepe (M)</t>
         </is>
       </c>
       <c r="Y94" t="n">
-        <v>620</v>
+        <v>140</v>
       </c>
       <c r="Z94" t="inlineStr">
         <is>
@@ -14176,11 +14212,23 @@
       </c>
       <c r="AA94" t="inlineStr"/>
       <c r="AB94" t="inlineStr"/>
-      <c r="AC94" t="inlineStr"/>
-      <c r="AD94" t="inlineStr"/>
-      <c r="AE94" t="inlineStr"/>
+      <c r="AC94" t="inlineStr">
+        <is>
+          <t>Gokul Texprints Pvt. Ltd. (Sachin)</t>
+        </is>
+      </c>
+      <c r="AD94" t="inlineStr">
+        <is>
+          <t>RVI-2627/07568</t>
+        </is>
+      </c>
+      <c r="AE94" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="AF94" t="n">
-        <v>0</v>
+        <v>144.5</v>
       </c>
       <c r="AG94" t="inlineStr"/>
       <c r="AH94" t="inlineStr"/>
@@ -14214,7 +14262,9 @@
       <c r="AV94" t="inlineStr"/>
       <c r="AW94" t="inlineStr"/>
       <c r="AX94" t="inlineStr"/>
-      <c r="AY94" t="inlineStr"/>
+      <c r="AY94" t="n">
+        <v>2</v>
+      </c>
       <c r="AZ94" t="inlineStr"/>
       <c r="BA94" t="inlineStr"/>
       <c r="BB94" t="inlineStr"/>
@@ -14222,16 +14272,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Modi Sons</t>
+          <t>Manisha Fabrics (Raipur)</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>['PSO-2627/04108']</t>
+          <t>['PSO-2627/04107']</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -14244,7 +14294,7 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>200</v>
+        <v>620</v>
       </c>
       <c r="G95" t="n">
         <v>0</v>
@@ -14279,7 +14329,7 @@
       </c>
       <c r="V95" t="inlineStr">
         <is>
-          <t>PJO-2627/04515</t>
+          <t>PJO-2627/04513-1</t>
         </is>
       </c>
       <c r="W95" t="inlineStr">
@@ -14293,7 +14343,7 @@
         </is>
       </c>
       <c r="Y95" t="n">
-        <v>200</v>
+        <v>620</v>
       </c>
       <c r="Z95" t="inlineStr">
         <is>
@@ -14348,36 +14398,36 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Chitrangana Fabrics</t>
+          <t>Modi Sons</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>['RSO-2627/01039']</t>
+          <t>['PSO-2627/04108']</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>10000</v>
+        <v>200</v>
       </c>
       <c r="G96" t="n">
-        <v>3657.75</v>
+        <v>0</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Jaipur</t>
+          <t>Raipur</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -14387,7 +14437,7 @@
         </is>
       </c>
       <c r="K96" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr"/>
@@ -14403,13 +14453,29 @@
       <c r="U96" t="n">
         <v>0</v>
       </c>
-      <c r="V96" t="inlineStr"/>
-      <c r="W96" t="inlineStr"/>
-      <c r="X96" t="inlineStr"/>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>PJO-2627/04515</t>
+        </is>
+      </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>RFD-Satin Bemberg New</t>
+        </is>
+      </c>
       <c r="Y96" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z96" t="inlineStr"/>
+        <v>200</v>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="AA96" t="inlineStr"/>
       <c r="AB96" t="inlineStr"/>
       <c r="AC96" t="inlineStr"/>
@@ -14426,28 +14492,12 @@
       <c r="AJ96" t="inlineStr"/>
       <c r="AK96" t="inlineStr"/>
       <c r="AL96" t="inlineStr"/>
-      <c r="AM96" t="inlineStr">
-        <is>
-          <t>RSD-2627/01479,RSD-2627/01409</t>
-        </is>
-      </c>
-      <c r="AN96" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="AO96" t="inlineStr">
-        <is>
-          <t>RSI-2627/01463,RSI-2627/01393</t>
-        </is>
-      </c>
-      <c r="AP96" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
+      <c r="AM96" t="inlineStr"/>
+      <c r="AN96" t="inlineStr"/>
+      <c r="AO96" t="inlineStr"/>
+      <c r="AP96" t="inlineStr"/>
       <c r="AQ96" t="n">
-        <v>3657.75</v>
+        <v>0</v>
       </c>
       <c r="AR96" t="inlineStr">
         <is>
@@ -14460,35 +14510,61 @@
           <t>Bikash Behera</t>
         </is>
       </c>
-      <c r="AU96" t="inlineStr"/>
+      <c r="AU96" t="n">
+        <v>0</v>
+      </c>
       <c r="AV96" t="inlineStr"/>
       <c r="AW96" t="inlineStr"/>
       <c r="AX96" t="inlineStr"/>
       <c r="AY96" t="inlineStr"/>
       <c r="AZ96" t="inlineStr"/>
-      <c r="BA96" t="n">
-        <v>30</v>
-      </c>
-      <c r="BB96" t="n">
-        <v>0</v>
-      </c>
+      <c r="BA96" t="inlineStr"/>
+      <c r="BB96" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr"/>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Chitrangana Fabrics</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>['RSO-2627/01039']</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>32</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="F97" t="n">
-        <v>55618</v>
+        <v>10000</v>
       </c>
       <c r="G97" t="n">
-        <v>11631.25</v>
-      </c>
-      <c r="H97" t="inlineStr"/>
+        <v>3657.75</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Jaipur</t>
+        </is>
+      </c>
       <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Bikash Behera</t>
+        </is>
+      </c>
+      <c r="K97" t="n">
+        <v>10</v>
+      </c>
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr"/>
       <c r="N97" t="inlineStr"/>
@@ -14507,7 +14583,7 @@
       <c r="W97" t="inlineStr"/>
       <c r="X97" t="inlineStr"/>
       <c r="Y97" t="n">
-        <v>42751</v>
+        <v>0</v>
       </c>
       <c r="Z97" t="inlineStr"/>
       <c r="AA97" t="inlineStr"/>
@@ -14516,34 +14592,242 @@
       <c r="AD97" t="inlineStr"/>
       <c r="AE97" t="inlineStr"/>
       <c r="AF97" t="n">
-        <v>31048.5</v>
+        <v>0</v>
       </c>
       <c r="AG97" t="inlineStr"/>
       <c r="AH97" t="inlineStr"/>
       <c r="AI97" t="n">
-        <v>13472.3</v>
+        <v>0</v>
       </c>
       <c r="AJ97" t="inlineStr"/>
       <c r="AK97" t="inlineStr"/>
       <c r="AL97" t="inlineStr"/>
-      <c r="AM97" t="inlineStr"/>
-      <c r="AN97" t="inlineStr"/>
-      <c r="AO97" t="inlineStr"/>
-      <c r="AP97" t="inlineStr"/>
+      <c r="AM97" t="inlineStr">
+        <is>
+          <t>RSD-2627/01479,RSD-2627/01409</t>
+        </is>
+      </c>
+      <c r="AN97" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="AO97" t="inlineStr">
+        <is>
+          <t>RSI-2627/01463,RSI-2627/01393</t>
+        </is>
+      </c>
+      <c r="AP97" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
       <c r="AQ97" t="n">
-        <v>11631.25</v>
-      </c>
-      <c r="AR97" t="inlineStr"/>
+        <v>3657.75</v>
+      </c>
+      <c r="AR97" t="inlineStr">
+        <is>
+          <t>To Deliver and Bill</t>
+        </is>
+      </c>
       <c r="AS97" t="inlineStr"/>
-      <c r="AT97" t="inlineStr"/>
+      <c r="AT97" t="inlineStr">
+        <is>
+          <t>Bikash Behera</t>
+        </is>
+      </c>
       <c r="AU97" t="inlineStr"/>
       <c r="AV97" t="inlineStr"/>
       <c r="AW97" t="inlineStr"/>
       <c r="AX97" t="inlineStr"/>
       <c r="AY97" t="inlineStr"/>
       <c r="AZ97" t="inlineStr"/>
-      <c r="BA97" t="inlineStr"/>
-      <c r="BB97" t="inlineStr"/>
+      <c r="BA97" t="n">
+        <v>30</v>
+      </c>
+      <c r="BB97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Meenakshi Wholesale &amp; Retail Fabrics</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>['RSO-2627/01243']</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>0</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>200</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Bikash Behera</t>
+        </is>
+      </c>
+      <c r="K98" t="n">
+        <v>2</v>
+      </c>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr"/>
+      <c r="P98" t="inlineStr"/>
+      <c r="Q98" t="inlineStr"/>
+      <c r="R98" t="n">
+        <v>0</v>
+      </c>
+      <c r="S98" t="inlineStr"/>
+      <c r="T98" t="inlineStr"/>
+      <c r="U98" t="n">
+        <v>0</v>
+      </c>
+      <c r="V98" t="inlineStr"/>
+      <c r="W98" t="inlineStr"/>
+      <c r="X98" t="inlineStr"/>
+      <c r="Y98" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z98" t="inlineStr"/>
+      <c r="AA98" t="inlineStr"/>
+      <c r="AB98" t="inlineStr"/>
+      <c r="AC98" t="inlineStr"/>
+      <c r="AD98" t="inlineStr"/>
+      <c r="AE98" t="inlineStr"/>
+      <c r="AF98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG98" t="inlineStr"/>
+      <c r="AH98" t="inlineStr"/>
+      <c r="AI98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ98" t="inlineStr"/>
+      <c r="AK98" t="inlineStr"/>
+      <c r="AL98" t="inlineStr"/>
+      <c r="AM98" t="inlineStr"/>
+      <c r="AN98" t="inlineStr"/>
+      <c r="AO98" t="inlineStr"/>
+      <c r="AP98" t="inlineStr"/>
+      <c r="AQ98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR98" t="inlineStr">
+        <is>
+          <t>To Deliver and Bill</t>
+        </is>
+      </c>
+      <c r="AS98" t="inlineStr"/>
+      <c r="AT98" t="inlineStr">
+        <is>
+          <t>Bikash Behera</t>
+        </is>
+      </c>
+      <c r="AU98" t="inlineStr"/>
+      <c r="AV98" t="inlineStr"/>
+      <c r="AW98" t="inlineStr"/>
+      <c r="AX98" t="inlineStr"/>
+      <c r="AY98" t="inlineStr"/>
+      <c r="AZ98" t="inlineStr"/>
+      <c r="BA98" t="inlineStr"/>
+      <c r="BB98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr"/>
+      <c r="B99" t="inlineStr"/>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="n">
+        <v>56463</v>
+      </c>
+      <c r="G99" t="n">
+        <v>12288.25</v>
+      </c>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr"/>
+      <c r="P99" t="inlineStr"/>
+      <c r="Q99" t="inlineStr"/>
+      <c r="R99" t="n">
+        <v>0</v>
+      </c>
+      <c r="S99" t="inlineStr"/>
+      <c r="T99" t="inlineStr"/>
+      <c r="U99" t="n">
+        <v>0</v>
+      </c>
+      <c r="V99" t="inlineStr"/>
+      <c r="W99" t="inlineStr"/>
+      <c r="X99" t="inlineStr"/>
+      <c r="Y99" t="n">
+        <v>42751</v>
+      </c>
+      <c r="Z99" t="inlineStr"/>
+      <c r="AA99" t="inlineStr"/>
+      <c r="AB99" t="inlineStr"/>
+      <c r="AC99" t="inlineStr"/>
+      <c r="AD99" t="inlineStr"/>
+      <c r="AE99" t="inlineStr"/>
+      <c r="AF99" t="n">
+        <v>31193</v>
+      </c>
+      <c r="AG99" t="inlineStr"/>
+      <c r="AH99" t="inlineStr"/>
+      <c r="AI99" t="n">
+        <v>13472.3</v>
+      </c>
+      <c r="AJ99" t="inlineStr"/>
+      <c r="AK99" t="inlineStr"/>
+      <c r="AL99" t="inlineStr"/>
+      <c r="AM99" t="inlineStr"/>
+      <c r="AN99" t="inlineStr"/>
+      <c r="AO99" t="inlineStr"/>
+      <c r="AP99" t="inlineStr"/>
+      <c r="AQ99" t="n">
+        <v>11631.25</v>
+      </c>
+      <c r="AR99" t="inlineStr"/>
+      <c r="AS99" t="inlineStr"/>
+      <c r="AT99" t="inlineStr"/>
+      <c r="AU99" t="inlineStr"/>
+      <c r="AV99" t="inlineStr"/>
+      <c r="AW99" t="inlineStr"/>
+      <c r="AX99" t="inlineStr"/>
+      <c r="AY99" t="inlineStr"/>
+      <c r="AZ99" t="inlineStr"/>
+      <c r="BA99" t="inlineStr"/>
+      <c r="BB99" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>